<commit_message>
Corrige acentuação corrompida nos municípios
</commit_message>
<xml_diff>
--- a/Dados_Precos.xlsx
+++ b/Dados_Precos.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ÃÂÃÂÃÂÃÂgua Clara</t>
+          <t>Água Clara</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -483,7 +483,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ÃÂÃÂgua Clara</t>
+          <t>Água Clara</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -503,7 +503,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ÃÂgua Clara</t>
+          <t>Água Clara</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -523,7 +523,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ÃÂgua Clara</t>
+          <t>Água Clara</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -543,7 +543,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ÃÂgua Clara</t>
+          <t>Água Clara</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -563,7 +563,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ÃÂgua Clara</t>
+          <t>Água Clara</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -583,7 +583,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ÃÂgua Clara</t>
+          <t>Água Clara</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -603,7 +603,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ãgua Clara</t>
+          <t>Água Clara</t>
         </is>
       </c>
       <c r="D9" t="n">

</xml_diff>

<commit_message>
Coleta de preços — 2026-07-10
</commit_message>
<xml_diff>
--- a/Dados_Precos.xlsx
+++ b/Dados_Precos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -630,6 +630,326 @@
         <v>109</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Raphael</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Água Clara</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>